<commit_message>
feat(fase-3): implementar agente orquestador con inteligencia artificial gemini y herramientas de analisis
</commit_message>
<xml_diff>
--- a/datos/NIT.xlsx
+++ b/datos/NIT.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4bb26ee33b2391af/Maestria inteligencia artificial/Tesis/Prototipo Sistema Agentes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4bb26ee33b2391af/Maestria inteligencia artificial/Tesis/Prototipo Sistema Agentes/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC10483F795B5FE45ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7DE8320-15CD-4A02-A549-4A906890A6A5}"/>

</xml_diff>